<commit_message>
Revisión de lenguaje: propuestas aprobadas (jefaturas, Administración, Accesos, Colegio, Mayor valoración primero, rangos sin partir en la web), mensajes del servidor con su migración, plantilla de asignación, especificación y documentación
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etl/plantillas/asignacion_docente_2526.xlsx
+++ b/etl/plantillas/asignacion_docente_2526.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Asignación" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Listas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asignación" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Asignación'!$A$1:$G$1</definedName>
@@ -463,7 +463,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Asignación de profesores por grupo y asignatura · curso 2025/26</t>
+          <t>Asignación docente por grupo y asignatura · curso 2025/26</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr"/>
@@ -480,7 +480,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Con esta tabla la plataforma de encuestas sabe qué docente imparte cada asignatura en cada grupo, para preparar el informe de cada profesor con las encuestas de sus alumnos.</t>
+          <t>Con esta tabla la plataforma de encuestas sabe qué docente imparte cada asignatura en cada grupo, para preparar el informe de cada profesor/a con las encuestas de su alumnado.</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Grupo de alumnos tal como aparece en la hoja Listas, por ejemplo «Y9 A».</t>
+          <t>Grupo tal como aparece en la hoja Listas, por ejemplo «Y9 A».</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Departamento al que pertenece el docente (para los informes de jefes de departamento).</t>
+          <t>Departamento al que pertenece el docente (para los informes de las jefaturas de departamento).</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Esta tabla solo se usa para atribuir los resultados agregados de las encuestas. Los alumnos no aparecen en ella y ningún resultado con menos de 5 respuestas se muestra en los informes.</t>
+          <t>Esta tabla solo se usa para atribuir los resultados agregados de las encuestas. El alumnado no aparece en ella y ningún resultado con menos de 5 respuestas se muestra en los informes.</t>
         </is>
       </c>
     </row>

</xml_diff>